<commit_message>
Updated Depeche Mod songs json
</commit_message>
<xml_diff>
--- a/data/Depeche Mode Songs.xlsx
+++ b/data/Depeche Mode Songs.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lindanakasone/Documents/GitHub/sound-and-vision/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{954E7000-B2BB-FC4A-9CD8-84C3922F8D00}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57A9EE82-772C-5B4A-9411-8B0DB45E8057}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1620" yWindow="4840" windowWidth="28040" windowHeight="22780" xr2:uid="{FE581154-A771-454D-BC0C-F4CC813A6F29}"/>
+    <workbookView xWindow="19780" yWindow="4760" windowWidth="28040" windowHeight="22780" xr2:uid="{FE581154-A771-454D-BC0C-F4CC813A6F29}"/>
   </bookViews>
   <sheets>
     <sheet name="Depeche Mode Songs" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="736" uniqueCount="280">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="739" uniqueCount="282">
   <si>
     <t>Song</t>
   </si>
@@ -259,9 +259,6 @@
     <t>Stripped</t>
   </si>
   <si>
-    <t>Here Is The House</t>
-  </si>
-  <si>
     <t>World Full Of Nothing</t>
   </si>
   <si>
@@ -394,18 +391,6 @@
     <t>Policy of Truth</t>
   </si>
   <si>
-    <t>Dangerous (Bonus Track)</t>
-  </si>
-  <si>
-    <t>Memphisto (Bonus Track)</t>
-  </si>
-  <si>
-    <t>Sibeling (Bonus Track)</t>
-  </si>
-  <si>
-    <t>Kaleid (Bonus Track)</t>
-  </si>
-  <si>
     <t>Barrel of a Gun</t>
   </si>
   <si>
@@ -863,6 +848,27 @@
   </si>
   <si>
     <t>Dave Gahan (age 46); Christian Eigner; Andrew Phillpott</t>
+  </si>
+  <si>
+    <t>Dangerous</t>
+  </si>
+  <si>
+    <t>Memphisto</t>
+  </si>
+  <si>
+    <t>Sibeling</t>
+  </si>
+  <si>
+    <t>Kaleid</t>
+  </si>
+  <si>
+    <t>A Question of Time</t>
+  </si>
+  <si>
+    <t>Here Is the House</t>
+  </si>
+  <si>
+    <t>Sea of Sin</t>
   </si>
 </sst>
 </file>
@@ -1738,7 +1744,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DE1C0B07-670E-FB45-A921-EAB11111294F}">
-  <dimension ref="A1:G245"/>
+  <dimension ref="A1:G246"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="37.83203125" customWidth="1"/>
@@ -1758,7 +1764,7 @@
         <v>3</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>4</v>
@@ -2453,7 +2459,7 @@
         <v>7</v>
       </c>
       <c r="F50" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.2">
@@ -2470,7 +2476,7 @@
         <v>7</v>
       </c>
       <c r="F51" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.2">
@@ -2487,7 +2493,7 @@
         <v>7</v>
       </c>
       <c r="F52" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.2">
@@ -2504,7 +2510,7 @@
         <v>24</v>
       </c>
       <c r="F53" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.2">
@@ -2521,7 +2527,7 @@
         <v>14</v>
       </c>
       <c r="F54" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.2">
@@ -2552,7 +2558,7 @@
         <v>33</v>
       </c>
       <c r="F56" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.2">
@@ -2569,7 +2575,7 @@
         <v>33</v>
       </c>
       <c r="F57" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.2">
@@ -2586,7 +2592,7 @@
         <v>60</v>
       </c>
       <c r="F58" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.2">
@@ -2603,7 +2609,7 @@
         <v>60</v>
       </c>
       <c r="F59" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.2">
@@ -2620,7 +2626,7 @@
         <v>60</v>
       </c>
       <c r="F60" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.2">
@@ -2637,7 +2643,7 @@
         <v>60</v>
       </c>
       <c r="F61" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.2">
@@ -2665,7 +2671,7 @@
         <v>1986</v>
       </c>
       <c r="D63" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.2">
@@ -2679,7 +2685,7 @@
         <v>1986</v>
       </c>
       <c r="D64" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.2">
@@ -2693,7 +2699,7 @@
         <v>1986</v>
       </c>
       <c r="D65" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.2">
@@ -2707,7 +2713,7 @@
         <v>1986</v>
       </c>
       <c r="D66" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.2">
@@ -2721,7 +2727,7 @@
         <v>1986</v>
       </c>
       <c r="D67" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.2">
@@ -2735,7 +2741,7 @@
         <v>1986</v>
       </c>
       <c r="D68" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.2">
@@ -2749,12 +2755,12 @@
         <v>1986</v>
       </c>
       <c r="D69" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
-        <v>78</v>
+        <v>280</v>
       </c>
       <c r="B70" t="s">
         <v>71</v>
@@ -2763,12 +2769,12 @@
         <v>1986</v>
       </c>
       <c r="D70" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B71" t="s">
         <v>71</v>
@@ -2777,12 +2783,12 @@
         <v>1986</v>
       </c>
       <c r="D71" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B72" t="s">
         <v>71</v>
@@ -2791,12 +2797,12 @@
         <v>1986</v>
       </c>
       <c r="D72" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B73" t="s">
         <v>71</v>
@@ -2805,12 +2811,12 @@
         <v>1986</v>
       </c>
       <c r="D73" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B74" t="s">
         <v>71</v>
@@ -2819,12 +2825,12 @@
         <v>1986</v>
       </c>
       <c r="D74" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B75" t="s">
         <v>71</v>
@@ -2833,12 +2839,12 @@
         <v>1986</v>
       </c>
       <c r="D75" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B76" t="s">
         <v>71</v>
@@ -2847,242 +2853,242 @@
         <v>1986</v>
       </c>
       <c r="D76" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B77" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C77">
         <v>1987</v>
       </c>
       <c r="D77" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B78" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C78">
         <v>1987</v>
       </c>
       <c r="D78" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B79" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C79">
         <v>1987</v>
       </c>
       <c r="D79" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B80" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C80">
         <v>1987</v>
       </c>
       <c r="D80" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="81" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B81" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C81">
         <v>1987</v>
       </c>
       <c r="D81" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="82" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B82" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C82">
         <v>1987</v>
       </c>
       <c r="D82" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="83" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B83" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C83">
         <v>1987</v>
       </c>
       <c r="D83" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="84" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B84" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C84">
         <v>1987</v>
       </c>
       <c r="D84" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="85" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B85" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C85">
         <v>1987</v>
       </c>
       <c r="D85" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="86" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B86" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C86">
         <v>1987</v>
       </c>
       <c r="D86" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="87" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B87" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C87">
         <v>1987</v>
       </c>
       <c r="D87" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="88" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B88" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C88">
         <v>1987</v>
       </c>
       <c r="D88" t="s">
+        <v>102</v>
+      </c>
+      <c r="G88" t="s">
         <v>103</v>
-      </c>
-      <c r="G88" t="s">
-        <v>104</v>
       </c>
     </row>
     <row r="89" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B89" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C89">
         <v>1987</v>
       </c>
       <c r="D89" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="G89" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="90" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
+        <v>98</v>
+      </c>
+      <c r="B90" t="s">
         <v>99</v>
-      </c>
-      <c r="B90" t="s">
-        <v>100</v>
       </c>
       <c r="C90">
         <v>1987</v>
       </c>
       <c r="D90" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="91" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A91" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B91" s="2">
         <v>101</v>
       </c>
       <c r="F91" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="92" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A92" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B92" s="2">
         <v>101</v>
       </c>
       <c r="F92" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="93" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A93" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B93" s="2">
         <v>101</v>
       </c>
       <c r="F93" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="94" spans="1:7" x14ac:dyDescent="0.2">
@@ -3093,7 +3099,7 @@
         <v>101</v>
       </c>
       <c r="F94" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="95" spans="1:7" x14ac:dyDescent="0.2">
@@ -3104,7 +3110,7 @@
         <v>101</v>
       </c>
       <c r="F95" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="96" spans="1:7" x14ac:dyDescent="0.2">
@@ -3115,7 +3121,7 @@
         <v>101</v>
       </c>
       <c r="F96" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="97" spans="1:6" x14ac:dyDescent="0.2">
@@ -3126,18 +3132,18 @@
         <v>101</v>
       </c>
       <c r="F97" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="98" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A98" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B98" s="2">
         <v>101</v>
       </c>
       <c r="F98" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="99" spans="1:6" x14ac:dyDescent="0.2">
@@ -3148,7 +3154,7 @@
         <v>101</v>
       </c>
       <c r="F99" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="100" spans="1:6" x14ac:dyDescent="0.2">
@@ -3159,12 +3165,12 @@
         <v>101</v>
       </c>
       <c r="F100" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="101" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A101" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B101" s="2">
         <v>101</v>
@@ -3173,10 +3179,10 @@
         <v>1987</v>
       </c>
       <c r="D101" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F101" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="102" spans="1:6" x14ac:dyDescent="0.2">
@@ -3187,29 +3193,29 @@
         <v>101</v>
       </c>
       <c r="F102" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="103" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A103" t="s">
-        <v>76</v>
+        <v>279</v>
       </c>
       <c r="B103" s="2">
         <v>101</v>
       </c>
       <c r="F103" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="104" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A104" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B104" s="2">
         <v>101</v>
       </c>
       <c r="F104" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="105" spans="1:6" x14ac:dyDescent="0.2">
@@ -3220,7 +3226,7 @@
         <v>101</v>
       </c>
       <c r="F105" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="106" spans="1:6" x14ac:dyDescent="0.2">
@@ -3231,7 +3237,7 @@
         <v>101</v>
       </c>
       <c r="F106" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="107" spans="1:6" x14ac:dyDescent="0.2">
@@ -3242,1939 +3248,1953 @@
         <v>101</v>
       </c>
       <c r="F107" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="108" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A108" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B108" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C108">
         <v>1990</v>
       </c>
       <c r="D108" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="109" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A109" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B109" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C109">
         <v>1990</v>
       </c>
       <c r="D109" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="110" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A110" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B110" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C110">
         <v>1989</v>
       </c>
       <c r="D110" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="111" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A111" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B111" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C111">
         <v>1990</v>
       </c>
       <c r="D111" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="112" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A112" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B112" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C112">
         <v>1990</v>
       </c>
       <c r="D112" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="113" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A113" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B113" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C113">
         <v>1990</v>
       </c>
       <c r="D113" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="114" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A114" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B114" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C114">
         <v>1990</v>
       </c>
       <c r="D114" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="115" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A115" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B115" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C115">
         <v>1990</v>
       </c>
       <c r="D115" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="116" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A116" t="s">
+        <v>116</v>
+      </c>
+      <c r="B116" t="s">
         <v>117</v>
-      </c>
-      <c r="B116" t="s">
-        <v>118</v>
       </c>
       <c r="C116">
         <v>1990</v>
       </c>
       <c r="D116" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="117" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A117" t="s">
-        <v>123</v>
+        <v>275</v>
       </c>
       <c r="B117" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C117">
         <v>1990</v>
       </c>
       <c r="D117" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="118" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A118" t="s">
-        <v>124</v>
+        <v>276</v>
       </c>
       <c r="B118" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C118">
         <v>1990</v>
       </c>
       <c r="D118" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="119" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A119" t="s">
-        <v>125</v>
+        <v>277</v>
       </c>
       <c r="B119" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C119">
         <v>1990</v>
       </c>
       <c r="D119" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="120" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A120" t="s">
-        <v>126</v>
+        <v>278</v>
       </c>
       <c r="B120" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C120">
         <v>1990</v>
       </c>
       <c r="D120" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="121" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A121" t="s">
-        <v>146</v>
+        <v>281</v>
       </c>
       <c r="B121" t="s">
-        <v>164</v>
+        <v>117</v>
       </c>
       <c r="C121">
-        <v>1993</v>
+        <v>1990</v>
       </c>
       <c r="D121" t="s">
-        <v>165</v>
+        <v>118</v>
       </c>
     </row>
     <row r="122" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A122" t="s">
-        <v>147</v>
+        <v>141</v>
       </c>
       <c r="B122" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
       <c r="C122">
         <v>1993</v>
       </c>
       <c r="D122" t="s">
-        <v>165</v>
+        <v>160</v>
       </c>
     </row>
     <row r="123" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A123" t="s">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="B123" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
       <c r="C123">
         <v>1993</v>
       </c>
       <c r="D123" t="s">
-        <v>165</v>
+        <v>160</v>
       </c>
     </row>
     <row r="124" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A124" t="s">
-        <v>149</v>
+        <v>143</v>
       </c>
       <c r="B124" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
       <c r="C124">
         <v>1993</v>
       </c>
       <c r="D124" t="s">
-        <v>165</v>
+        <v>160</v>
       </c>
     </row>
     <row r="125" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A125" t="s">
-        <v>150</v>
+        <v>144</v>
       </c>
       <c r="B125" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
       <c r="C125">
         <v>1993</v>
       </c>
       <c r="D125" t="s">
-        <v>165</v>
+        <v>160</v>
       </c>
     </row>
     <row r="126" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A126" t="s">
-        <v>151</v>
+        <v>145</v>
       </c>
       <c r="B126" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
       <c r="C126">
         <v>1993</v>
       </c>
       <c r="D126" t="s">
-        <v>165</v>
+        <v>160</v>
       </c>
     </row>
     <row r="127" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A127" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="B127" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
       <c r="C127">
         <v>1993</v>
       </c>
       <c r="D127" t="s">
-        <v>165</v>
+        <v>160</v>
       </c>
     </row>
     <row r="128" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A128" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="B128" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
       <c r="C128">
         <v>1993</v>
       </c>
       <c r="D128" t="s">
-        <v>165</v>
+        <v>160</v>
       </c>
     </row>
     <row r="129" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A129" t="s">
-        <v>154</v>
+        <v>148</v>
       </c>
       <c r="B129" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
       <c r="C129">
         <v>1993</v>
       </c>
       <c r="D129" t="s">
-        <v>165</v>
+        <v>160</v>
       </c>
     </row>
     <row r="130" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A130" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
       <c r="B130" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
       <c r="C130">
         <v>1993</v>
       </c>
       <c r="D130" t="s">
-        <v>165</v>
+        <v>160</v>
       </c>
     </row>
     <row r="131" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A131" t="s">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="B131" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
       <c r="C131">
         <v>1993</v>
       </c>
       <c r="D131" t="s">
-        <v>165</v>
+        <v>160</v>
       </c>
     </row>
     <row r="132" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A132" t="s">
-        <v>157</v>
+        <v>151</v>
       </c>
       <c r="B132" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
       <c r="C132">
         <v>1993</v>
       </c>
       <c r="D132" t="s">
-        <v>165</v>
+        <v>160</v>
       </c>
     </row>
     <row r="133" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A133" t="s">
-        <v>158</v>
+        <v>152</v>
       </c>
       <c r="B133" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
       <c r="C133">
         <v>1993</v>
       </c>
       <c r="D133" t="s">
-        <v>165</v>
+        <v>160</v>
       </c>
     </row>
     <row r="134" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A134" t="s">
+        <v>153</v>
+      </c>
+      <c r="B134" t="s">
         <v>159</v>
-      </c>
-      <c r="B134" t="s">
-        <v>164</v>
       </c>
       <c r="C134">
         <v>1993</v>
       </c>
       <c r="D134" t="s">
-        <v>165</v>
+        <v>160</v>
       </c>
     </row>
     <row r="135" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A135" t="s">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="B135" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
       <c r="C135">
         <v>1993</v>
       </c>
       <c r="D135" t="s">
-        <v>165</v>
+        <v>160</v>
       </c>
     </row>
     <row r="136" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A136" t="s">
-        <v>161</v>
+        <v>155</v>
       </c>
       <c r="B136" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
       <c r="C136">
         <v>1993</v>
       </c>
       <c r="D136" t="s">
-        <v>165</v>
+        <v>160</v>
       </c>
     </row>
     <row r="137" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A137" t="s">
-        <v>162</v>
+        <v>156</v>
       </c>
       <c r="B137" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
       <c r="C137">
         <v>1993</v>
       </c>
       <c r="D137" t="s">
-        <v>165</v>
+        <v>160</v>
       </c>
     </row>
     <row r="138" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A138" t="s">
-        <v>163</v>
+        <v>157</v>
       </c>
       <c r="B138" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
       <c r="C138">
         <v>1993</v>
       </c>
       <c r="D138" t="s">
-        <v>165</v>
+        <v>160</v>
       </c>
     </row>
     <row r="139" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A139" t="s">
-        <v>127</v>
+        <v>158</v>
       </c>
       <c r="B139" t="s">
-        <v>144</v>
+        <v>159</v>
       </c>
       <c r="C139">
-        <v>1997</v>
+        <v>1993</v>
       </c>
       <c r="D139" t="s">
-        <v>145</v>
+        <v>160</v>
       </c>
     </row>
     <row r="140" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A140" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
       <c r="B140" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
       <c r="C140">
         <v>1997</v>
       </c>
       <c r="D140" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
     </row>
     <row r="141" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A141" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="B141" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
       <c r="C141">
         <v>1997</v>
       </c>
       <c r="D141" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
     </row>
     <row r="142" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A142" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
       <c r="B142" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
       <c r="C142">
         <v>1997</v>
       </c>
       <c r="D142" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
     </row>
     <row r="143" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A143" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
       <c r="B143" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
       <c r="C143">
         <v>1997</v>
       </c>
       <c r="D143" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
     </row>
     <row r="144" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A144" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="B144" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
       <c r="C144">
         <v>1997</v>
       </c>
       <c r="D144" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
     </row>
     <row r="145" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A145" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="B145" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
       <c r="C145">
         <v>1997</v>
       </c>
       <c r="D145" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
     </row>
     <row r="146" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A146" t="s">
-        <v>134</v>
+        <v>128</v>
       </c>
       <c r="B146" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
       <c r="C146">
         <v>1997</v>
       </c>
       <c r="D146" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
     </row>
     <row r="147" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A147" t="s">
-        <v>135</v>
+        <v>129</v>
       </c>
       <c r="B147" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
       <c r="C147">
         <v>1997</v>
       </c>
       <c r="D147" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
     </row>
     <row r="148" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A148" t="s">
-        <v>136</v>
+        <v>130</v>
       </c>
       <c r="B148" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
       <c r="C148">
         <v>1997</v>
       </c>
       <c r="D148" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
     </row>
     <row r="149" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A149" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="B149" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
       <c r="C149">
         <v>1997</v>
       </c>
       <c r="D149" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
     </row>
     <row r="150" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A150" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
       <c r="B150" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
       <c r="C150">
         <v>1997</v>
       </c>
       <c r="D150" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
     </row>
     <row r="151" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A151" t="s">
+        <v>133</v>
+      </c>
+      <c r="B151" t="s">
         <v>139</v>
-      </c>
-      <c r="B151" t="s">
-        <v>144</v>
       </c>
       <c r="C151">
         <v>1997</v>
       </c>
       <c r="D151" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
     </row>
     <row r="152" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A152" t="s">
-        <v>140</v>
+        <v>134</v>
       </c>
       <c r="B152" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
       <c r="C152">
         <v>1997</v>
       </c>
       <c r="D152" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
     </row>
     <row r="153" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A153" t="s">
-        <v>141</v>
+        <v>135</v>
       </c>
       <c r="B153" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
       <c r="C153">
-        <v>1998</v>
+        <v>1997</v>
       </c>
       <c r="D153" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
     </row>
     <row r="154" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A154" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
       <c r="B154" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
       <c r="C154">
         <v>1998</v>
       </c>
       <c r="D154" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
     </row>
     <row r="155" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A155" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="B155" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
       <c r="C155">
         <v>1998</v>
       </c>
       <c r="D155" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
     </row>
     <row r="156" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A156" t="s">
-        <v>166</v>
+        <v>138</v>
       </c>
       <c r="B156" t="s">
-        <v>183</v>
+        <v>139</v>
       </c>
       <c r="C156">
-        <v>2001</v>
+        <v>1998</v>
       </c>
       <c r="D156" t="s">
-        <v>184</v>
+        <v>140</v>
       </c>
     </row>
     <row r="157" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A157" t="s">
-        <v>167</v>
+        <v>161</v>
       </c>
       <c r="B157" t="s">
-        <v>183</v>
+        <v>178</v>
       </c>
       <c r="C157">
         <v>2001</v>
       </c>
       <c r="D157" t="s">
-        <v>184</v>
+        <v>179</v>
       </c>
     </row>
     <row r="158" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A158" t="s">
-        <v>168</v>
+        <v>162</v>
       </c>
       <c r="B158" t="s">
-        <v>183</v>
+        <v>178</v>
       </c>
       <c r="C158">
         <v>2001</v>
       </c>
       <c r="D158" t="s">
-        <v>184</v>
+        <v>179</v>
       </c>
     </row>
     <row r="159" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A159" t="s">
-        <v>169</v>
+        <v>163</v>
       </c>
       <c r="B159" t="s">
-        <v>183</v>
+        <v>178</v>
       </c>
       <c r="C159">
         <v>2001</v>
       </c>
       <c r="D159" t="s">
-        <v>184</v>
+        <v>179</v>
       </c>
     </row>
     <row r="160" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A160" t="s">
-        <v>170</v>
+        <v>164</v>
       </c>
       <c r="B160" t="s">
-        <v>183</v>
+        <v>178</v>
       </c>
       <c r="C160">
         <v>2001</v>
       </c>
       <c r="D160" t="s">
-        <v>184</v>
+        <v>179</v>
       </c>
     </row>
     <row r="161" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A161" t="s">
-        <v>171</v>
+        <v>165</v>
       </c>
       <c r="B161" t="s">
-        <v>183</v>
+        <v>178</v>
       </c>
       <c r="C161">
         <v>2001</v>
       </c>
       <c r="D161" t="s">
-        <v>184</v>
+        <v>179</v>
       </c>
     </row>
     <row r="162" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A162" t="s">
-        <v>172</v>
+        <v>166</v>
       </c>
       <c r="B162" t="s">
-        <v>183</v>
+        <v>178</v>
       </c>
       <c r="C162">
         <v>2001</v>
       </c>
       <c r="D162" t="s">
-        <v>184</v>
+        <v>179</v>
       </c>
     </row>
     <row r="163" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A163" t="s">
-        <v>173</v>
+        <v>167</v>
       </c>
       <c r="B163" t="s">
-        <v>183</v>
+        <v>178</v>
       </c>
       <c r="C163">
         <v>2001</v>
       </c>
       <c r="D163" t="s">
-        <v>184</v>
+        <v>179</v>
       </c>
     </row>
     <row r="164" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A164" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
       <c r="B164" t="s">
-        <v>183</v>
+        <v>178</v>
       </c>
       <c r="C164">
         <v>2001</v>
       </c>
       <c r="D164" t="s">
-        <v>184</v>
+        <v>179</v>
       </c>
     </row>
     <row r="165" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A165" t="s">
-        <v>175</v>
+        <v>169</v>
       </c>
       <c r="B165" t="s">
-        <v>183</v>
+        <v>178</v>
       </c>
       <c r="C165">
         <v>2001</v>
       </c>
       <c r="D165" t="s">
-        <v>184</v>
+        <v>179</v>
       </c>
     </row>
     <row r="166" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A166" t="s">
-        <v>176</v>
+        <v>170</v>
       </c>
       <c r="B166" t="s">
-        <v>183</v>
+        <v>178</v>
       </c>
       <c r="C166">
         <v>2001</v>
       </c>
       <c r="D166" t="s">
-        <v>184</v>
+        <v>179</v>
       </c>
     </row>
     <row r="167" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A167" t="s">
-        <v>177</v>
+        <v>171</v>
       </c>
       <c r="B167" t="s">
-        <v>183</v>
+        <v>178</v>
       </c>
       <c r="C167">
         <v>2001</v>
       </c>
       <c r="D167" t="s">
-        <v>184</v>
+        <v>179</v>
       </c>
     </row>
     <row r="168" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A168" t="s">
+        <v>172</v>
+      </c>
+      <c r="B168" t="s">
         <v>178</v>
-      </c>
-      <c r="B168" t="s">
-        <v>183</v>
       </c>
       <c r="C168">
         <v>2001</v>
       </c>
       <c r="D168" t="s">
-        <v>184</v>
+        <v>179</v>
       </c>
     </row>
     <row r="169" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A169" t="s">
-        <v>179</v>
+        <v>173</v>
       </c>
       <c r="B169" t="s">
-        <v>183</v>
+        <v>178</v>
       </c>
       <c r="C169">
         <v>2001</v>
       </c>
       <c r="D169" t="s">
-        <v>184</v>
+        <v>179</v>
       </c>
     </row>
     <row r="170" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A170" t="s">
-        <v>180</v>
+        <v>174</v>
       </c>
       <c r="B170" t="s">
-        <v>183</v>
+        <v>178</v>
       </c>
       <c r="C170">
         <v>2001</v>
       </c>
       <c r="D170" t="s">
-        <v>184</v>
+        <v>179</v>
       </c>
     </row>
     <row r="171" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A171" t="s">
-        <v>181</v>
+        <v>175</v>
       </c>
       <c r="B171" t="s">
-        <v>183</v>
+        <v>178</v>
       </c>
       <c r="C171">
         <v>2001</v>
       </c>
       <c r="D171" t="s">
-        <v>184</v>
+        <v>179</v>
       </c>
     </row>
     <row r="172" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A172" t="s">
-        <v>182</v>
+        <v>176</v>
       </c>
       <c r="B172" t="s">
-        <v>183</v>
+        <v>178</v>
       </c>
       <c r="C172">
         <v>2001</v>
       </c>
       <c r="D172" t="s">
-        <v>184</v>
+        <v>179</v>
       </c>
     </row>
     <row r="173" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A173" t="s">
-        <v>185</v>
+        <v>177</v>
       </c>
       <c r="B173" t="s">
-        <v>186</v>
+        <v>178</v>
       </c>
       <c r="C173">
-        <v>2005</v>
+        <v>2001</v>
       </c>
       <c r="D173" t="s">
-        <v>198</v>
+        <v>179</v>
       </c>
     </row>
     <row r="174" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A174" t="s">
-        <v>187</v>
+        <v>180</v>
       </c>
       <c r="B174" t="s">
-        <v>186</v>
+        <v>181</v>
       </c>
       <c r="C174">
         <v>2005</v>
       </c>
       <c r="D174" t="s">
-        <v>198</v>
+        <v>193</v>
       </c>
     </row>
     <row r="175" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A175" t="s">
-        <v>188</v>
+        <v>182</v>
       </c>
       <c r="B175" t="s">
-        <v>186</v>
+        <v>181</v>
       </c>
       <c r="C175">
         <v>2005</v>
       </c>
       <c r="D175" t="s">
-        <v>199</v>
+        <v>193</v>
       </c>
     </row>
     <row r="176" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A176" t="s">
-        <v>189</v>
+        <v>183</v>
       </c>
       <c r="B176" t="s">
-        <v>186</v>
+        <v>181</v>
       </c>
       <c r="C176">
         <v>2005</v>
       </c>
       <c r="D176" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
     </row>
     <row r="177" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A177" t="s">
-        <v>190</v>
+        <v>184</v>
       </c>
       <c r="B177" t="s">
-        <v>186</v>
+        <v>181</v>
       </c>
       <c r="C177">
         <v>2005</v>
       </c>
       <c r="D177" t="s">
-        <v>198</v>
+        <v>193</v>
       </c>
     </row>
     <row r="178" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A178" t="s">
-        <v>191</v>
+        <v>185</v>
       </c>
       <c r="B178" t="s">
-        <v>186</v>
+        <v>181</v>
       </c>
       <c r="C178">
         <v>2005</v>
       </c>
       <c r="D178" t="s">
-        <v>198</v>
+        <v>193</v>
       </c>
     </row>
     <row r="179" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A179" t="s">
-        <v>192</v>
+        <v>186</v>
       </c>
       <c r="B179" t="s">
-        <v>186</v>
+        <v>181</v>
       </c>
       <c r="C179">
         <v>2005</v>
       </c>
       <c r="D179" t="s">
-        <v>199</v>
+        <v>193</v>
       </c>
     </row>
     <row r="180" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A180" t="s">
-        <v>193</v>
+        <v>187</v>
       </c>
       <c r="B180" t="s">
-        <v>186</v>
+        <v>181</v>
       </c>
       <c r="C180">
         <v>2005</v>
       </c>
       <c r="D180" t="s">
-        <v>199</v>
+        <v>194</v>
       </c>
     </row>
     <row r="181" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A181" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="B181" t="s">
-        <v>186</v>
+        <v>181</v>
       </c>
       <c r="C181">
         <v>2005</v>
       </c>
       <c r="D181" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
     </row>
     <row r="182" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A182" t="s">
-        <v>195</v>
+        <v>189</v>
       </c>
       <c r="B182" t="s">
-        <v>186</v>
+        <v>181</v>
       </c>
       <c r="C182">
         <v>2005</v>
       </c>
       <c r="D182" t="s">
-        <v>198</v>
+        <v>193</v>
       </c>
     </row>
     <row r="183" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A183" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="B183" t="s">
-        <v>186</v>
+        <v>181</v>
       </c>
       <c r="C183">
         <v>2005</v>
       </c>
       <c r="D183" t="s">
-        <v>198</v>
+        <v>193</v>
       </c>
     </row>
     <row r="184" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A184" t="s">
-        <v>197</v>
+        <v>191</v>
       </c>
       <c r="B184" t="s">
-        <v>186</v>
+        <v>181</v>
       </c>
       <c r="C184">
         <v>2005</v>
       </c>
       <c r="D184" t="s">
-        <v>198</v>
+        <v>193</v>
       </c>
     </row>
     <row r="185" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A185" t="s">
-        <v>200</v>
+        <v>192</v>
       </c>
       <c r="B185" t="s">
-        <v>202</v>
+        <v>181</v>
       </c>
       <c r="C185">
-        <v>2006</v>
+        <v>2005</v>
       </c>
       <c r="D185" t="s">
-        <v>201</v>
+        <v>193</v>
       </c>
     </row>
     <row r="186" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A186" t="s">
-        <v>203</v>
+        <v>195</v>
       </c>
       <c r="B186" t="s">
-        <v>221</v>
+        <v>197</v>
       </c>
       <c r="C186">
-        <v>2009</v>
+        <v>2006</v>
       </c>
       <c r="D186" t="s">
-        <v>222</v>
+        <v>196</v>
       </c>
     </row>
     <row r="187" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A187" t="s">
-        <v>204</v>
+        <v>198</v>
       </c>
       <c r="B187" t="s">
-        <v>221</v>
+        <v>216</v>
       </c>
       <c r="C187">
         <v>2009</v>
       </c>
       <c r="D187" t="s">
-        <v>279</v>
+        <v>217</v>
       </c>
     </row>
     <row r="188" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A188" t="s">
-        <v>205</v>
+        <v>199</v>
       </c>
       <c r="B188" t="s">
-        <v>221</v>
+        <v>216</v>
       </c>
       <c r="C188">
         <v>2009</v>
       </c>
       <c r="D188" t="s">
-        <v>222</v>
+        <v>274</v>
       </c>
     </row>
     <row r="189" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A189" t="s">
-        <v>206</v>
+        <v>200</v>
       </c>
       <c r="B189" t="s">
-        <v>221</v>
+        <v>216</v>
       </c>
       <c r="C189">
         <v>2009</v>
       </c>
       <c r="D189" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
     </row>
     <row r="190" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A190" t="s">
-        <v>207</v>
+        <v>201</v>
       </c>
       <c r="B190" t="s">
-        <v>221</v>
+        <v>216</v>
       </c>
       <c r="C190">
         <v>2009</v>
       </c>
       <c r="D190" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
     </row>
     <row r="191" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A191" t="s">
-        <v>208</v>
+        <v>202</v>
       </c>
       <c r="B191" t="s">
-        <v>221</v>
+        <v>216</v>
       </c>
       <c r="C191">
         <v>2009</v>
       </c>
       <c r="D191" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
     </row>
     <row r="192" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A192" t="s">
-        <v>209</v>
+        <v>203</v>
       </c>
       <c r="B192" t="s">
-        <v>221</v>
+        <v>216</v>
       </c>
       <c r="C192">
         <v>2009</v>
       </c>
       <c r="D192" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
     </row>
     <row r="193" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A193" t="s">
-        <v>210</v>
+        <v>204</v>
       </c>
       <c r="B193" t="s">
-        <v>221</v>
+        <v>216</v>
       </c>
       <c r="C193">
         <v>2009</v>
       </c>
       <c r="D193" t="s">
-        <v>279</v>
+        <v>217</v>
       </c>
     </row>
     <row r="194" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A194" t="s">
-        <v>211</v>
+        <v>205</v>
       </c>
       <c r="B194" t="s">
-        <v>221</v>
+        <v>216</v>
       </c>
       <c r="C194">
         <v>2009</v>
       </c>
       <c r="D194" t="s">
-        <v>222</v>
+        <v>274</v>
       </c>
     </row>
     <row r="195" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A195" t="s">
-        <v>212</v>
+        <v>206</v>
       </c>
       <c r="B195" t="s">
-        <v>221</v>
+        <v>216</v>
       </c>
       <c r="C195">
         <v>2009</v>
       </c>
       <c r="D195" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
     </row>
     <row r="196" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A196" t="s">
-        <v>213</v>
+        <v>207</v>
       </c>
       <c r="B196" t="s">
-        <v>221</v>
+        <v>216</v>
       </c>
       <c r="C196">
         <v>2009</v>
       </c>
       <c r="D196" t="s">
-        <v>279</v>
+        <v>217</v>
       </c>
     </row>
     <row r="197" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A197" t="s">
-        <v>214</v>
+        <v>208</v>
       </c>
       <c r="B197" t="s">
-        <v>221</v>
+        <v>216</v>
       </c>
       <c r="C197">
         <v>2009</v>
       </c>
       <c r="D197" t="s">
-        <v>222</v>
+        <v>274</v>
       </c>
     </row>
     <row r="198" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A198" t="s">
-        <v>215</v>
+        <v>209</v>
       </c>
       <c r="B198" t="s">
-        <v>221</v>
+        <v>216</v>
       </c>
       <c r="C198">
         <v>2009</v>
       </c>
       <c r="D198" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
     </row>
     <row r="199" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A199" t="s">
+        <v>210</v>
+      </c>
+      <c r="B199" t="s">
         <v>216</v>
-      </c>
-      <c r="B199" t="s">
-        <v>221</v>
       </c>
       <c r="C199">
         <v>2009</v>
       </c>
       <c r="D199" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
     </row>
     <row r="200" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A200" t="s">
-        <v>217</v>
+        <v>211</v>
       </c>
       <c r="B200" t="s">
-        <v>221</v>
+        <v>216</v>
       </c>
       <c r="C200">
         <v>2009</v>
       </c>
       <c r="D200" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
     </row>
     <row r="201" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A201" t="s">
-        <v>218</v>
+        <v>212</v>
       </c>
       <c r="B201" t="s">
-        <v>221</v>
+        <v>216</v>
       </c>
       <c r="C201">
         <v>2009</v>
       </c>
       <c r="D201" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
     </row>
     <row r="202" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A202" t="s">
-        <v>219</v>
+        <v>213</v>
       </c>
       <c r="B202" t="s">
-        <v>221</v>
+        <v>216</v>
       </c>
       <c r="C202">
         <v>2009</v>
       </c>
       <c r="D202" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
     </row>
     <row r="203" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A203" t="s">
-        <v>220</v>
+        <v>214</v>
       </c>
       <c r="B203" t="s">
-        <v>221</v>
+        <v>216</v>
       </c>
       <c r="C203">
         <v>2009</v>
       </c>
       <c r="D203" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
     </row>
     <row r="204" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A204" t="s">
-        <v>223</v>
+        <v>215</v>
       </c>
       <c r="B204" t="s">
-        <v>224</v>
+        <v>216</v>
       </c>
       <c r="C204">
-        <v>2013</v>
+        <v>2009</v>
       </c>
       <c r="D204" t="s">
-        <v>238</v>
+        <v>217</v>
       </c>
     </row>
     <row r="205" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A205" t="s">
-        <v>225</v>
+        <v>218</v>
       </c>
       <c r="B205" t="s">
-        <v>224</v>
+        <v>219</v>
       </c>
       <c r="C205">
         <v>2013</v>
       </c>
       <c r="D205" t="s">
-        <v>238</v>
+        <v>233</v>
       </c>
     </row>
     <row r="206" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A206" t="s">
-        <v>226</v>
+        <v>220</v>
       </c>
       <c r="B206" t="s">
-        <v>224</v>
+        <v>219</v>
       </c>
       <c r="C206">
         <v>2013</v>
       </c>
       <c r="D206" t="s">
-        <v>238</v>
+        <v>233</v>
       </c>
     </row>
     <row r="207" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A207" t="s">
-        <v>227</v>
+        <v>221</v>
       </c>
       <c r="B207" t="s">
-        <v>224</v>
+        <v>219</v>
       </c>
       <c r="C207">
         <v>2013</v>
       </c>
       <c r="D207" t="s">
-        <v>237</v>
+        <v>233</v>
       </c>
     </row>
     <row r="208" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A208" t="s">
-        <v>228</v>
+        <v>222</v>
       </c>
       <c r="B208" t="s">
-        <v>224</v>
+        <v>219</v>
       </c>
       <c r="C208">
         <v>2013</v>
       </c>
       <c r="D208" t="s">
-        <v>238</v>
+        <v>232</v>
       </c>
     </row>
     <row r="209" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A209" t="s">
-        <v>229</v>
+        <v>223</v>
       </c>
       <c r="B209" t="s">
-        <v>224</v>
+        <v>219</v>
       </c>
       <c r="C209">
         <v>2013</v>
       </c>
       <c r="D209" t="s">
-        <v>238</v>
+        <v>233</v>
       </c>
     </row>
     <row r="210" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A210" t="s">
-        <v>230</v>
+        <v>224</v>
       </c>
       <c r="B210" t="s">
-        <v>224</v>
+        <v>219</v>
       </c>
       <c r="C210">
         <v>2013</v>
       </c>
       <c r="D210" t="s">
-        <v>237</v>
+        <v>233</v>
       </c>
     </row>
     <row r="211" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A211" t="s">
-        <v>231</v>
+        <v>225</v>
       </c>
       <c r="B211" t="s">
-        <v>224</v>
+        <v>219</v>
       </c>
       <c r="C211">
         <v>2013</v>
       </c>
       <c r="D211" t="s">
-        <v>238</v>
+        <v>232</v>
       </c>
     </row>
     <row r="212" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A212" t="s">
-        <v>232</v>
+        <v>226</v>
       </c>
       <c r="B212" t="s">
-        <v>224</v>
+        <v>219</v>
       </c>
       <c r="C212">
         <v>2013</v>
       </c>
       <c r="D212" t="s">
-        <v>238</v>
+        <v>233</v>
       </c>
     </row>
     <row r="213" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A213" t="s">
-        <v>233</v>
+        <v>227</v>
       </c>
       <c r="B213" t="s">
-        <v>224</v>
+        <v>219</v>
       </c>
       <c r="C213">
         <v>2013</v>
       </c>
       <c r="D213" t="s">
-        <v>237</v>
+        <v>233</v>
       </c>
     </row>
     <row r="214" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A214" t="s">
-        <v>234</v>
+        <v>228</v>
       </c>
       <c r="B214" t="s">
-        <v>224</v>
+        <v>219</v>
       </c>
       <c r="C214">
         <v>2013</v>
       </c>
       <c r="D214" t="s">
-        <v>238</v>
+        <v>232</v>
       </c>
     </row>
     <row r="215" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A215" t="s">
-        <v>235</v>
+        <v>229</v>
       </c>
       <c r="B215" t="s">
-        <v>224</v>
+        <v>219</v>
       </c>
       <c r="C215">
         <v>2013</v>
       </c>
       <c r="D215" t="s">
-        <v>238</v>
+        <v>233</v>
       </c>
     </row>
     <row r="216" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A216" t="s">
-        <v>236</v>
+        <v>230</v>
       </c>
       <c r="B216" t="s">
-        <v>224</v>
+        <v>219</v>
       </c>
       <c r="C216">
         <v>2013</v>
       </c>
       <c r="D216" t="s">
-        <v>238</v>
+        <v>233</v>
       </c>
     </row>
     <row r="217" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A217" t="s">
-        <v>239</v>
+        <v>231</v>
       </c>
       <c r="B217" t="s">
-        <v>256</v>
+        <v>219</v>
       </c>
       <c r="C217">
-        <v>2017</v>
+        <v>2013</v>
       </c>
       <c r="D217" t="s">
-        <v>257</v>
+        <v>233</v>
       </c>
     </row>
     <row r="218" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A218" t="s">
-        <v>240</v>
+        <v>234</v>
       </c>
       <c r="B218" t="s">
-        <v>256</v>
+        <v>251</v>
       </c>
       <c r="C218">
         <v>2017</v>
       </c>
       <c r="D218" t="s">
-        <v>257</v>
+        <v>252</v>
       </c>
     </row>
     <row r="219" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A219" t="s">
-        <v>241</v>
+        <v>235</v>
       </c>
       <c r="B219" t="s">
-        <v>256</v>
+        <v>251</v>
       </c>
       <c r="C219">
         <v>2017</v>
       </c>
       <c r="D219" t="s">
-        <v>257</v>
+        <v>252</v>
       </c>
     </row>
     <row r="220" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A220" t="s">
-        <v>242</v>
+        <v>236</v>
       </c>
       <c r="B220" t="s">
-        <v>256</v>
+        <v>251</v>
       </c>
       <c r="C220">
         <v>2017</v>
       </c>
       <c r="D220" t="s">
-        <v>257</v>
+        <v>252</v>
       </c>
     </row>
     <row r="221" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A221" t="s">
-        <v>243</v>
+        <v>237</v>
       </c>
       <c r="B221" t="s">
-        <v>256</v>
+        <v>251</v>
       </c>
       <c r="C221">
         <v>2017</v>
       </c>
       <c r="D221" t="s">
-        <v>258</v>
+        <v>252</v>
       </c>
     </row>
     <row r="222" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A222" t="s">
-        <v>244</v>
+        <v>238</v>
       </c>
       <c r="B222" t="s">
-        <v>256</v>
+        <v>251</v>
       </c>
       <c r="C222">
         <v>2017</v>
       </c>
       <c r="D222" t="s">
-        <v>259</v>
+        <v>253</v>
       </c>
     </row>
     <row r="223" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A223" t="s">
-        <v>245</v>
+        <v>239</v>
       </c>
       <c r="B223" t="s">
-        <v>256</v>
+        <v>251</v>
       </c>
       <c r="C223">
         <v>2017</v>
       </c>
       <c r="D223" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
     </row>
     <row r="224" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A224" t="s">
-        <v>246</v>
+        <v>240</v>
       </c>
       <c r="B224" t="s">
-        <v>256</v>
+        <v>251</v>
       </c>
       <c r="C224">
         <v>2017</v>
       </c>
       <c r="D224" t="s">
-        <v>259</v>
+        <v>252</v>
       </c>
     </row>
     <row r="225" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A225" t="s">
-        <v>247</v>
+        <v>241</v>
       </c>
       <c r="B225" t="s">
-        <v>256</v>
+        <v>251</v>
       </c>
       <c r="C225">
         <v>2017</v>
       </c>
       <c r="D225" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
     </row>
     <row r="226" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A226" t="s">
-        <v>248</v>
+        <v>242</v>
       </c>
       <c r="B226" t="s">
-        <v>256</v>
+        <v>251</v>
       </c>
       <c r="C226">
         <v>2017</v>
       </c>
       <c r="D226" t="s">
-        <v>257</v>
+        <v>252</v>
       </c>
     </row>
     <row r="227" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A227" t="s">
-        <v>249</v>
+        <v>243</v>
       </c>
       <c r="B227" t="s">
-        <v>256</v>
+        <v>251</v>
       </c>
       <c r="C227">
         <v>2017</v>
       </c>
       <c r="D227" t="s">
-        <v>260</v>
+        <v>252</v>
       </c>
     </row>
     <row r="228" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A228" t="s">
-        <v>250</v>
+        <v>244</v>
       </c>
       <c r="B228" t="s">
-        <v>256</v>
+        <v>251</v>
       </c>
       <c r="C228">
         <v>2017</v>
       </c>
       <c r="D228" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
     </row>
     <row r="229" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A229" t="s">
+        <v>245</v>
+      </c>
+      <c r="B229" t="s">
         <v>251</v>
-      </c>
-      <c r="B229" t="s">
-        <v>256</v>
       </c>
       <c r="C229">
         <v>2017</v>
       </c>
       <c r="D229" t="s">
-        <v>257</v>
+        <v>252</v>
       </c>
     </row>
     <row r="230" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A230" t="s">
-        <v>252</v>
+        <v>246</v>
       </c>
       <c r="B230" t="s">
-        <v>256</v>
+        <v>251</v>
       </c>
       <c r="C230">
         <v>2017</v>
       </c>
       <c r="D230" t="s">
-        <v>257</v>
+        <v>252</v>
       </c>
     </row>
     <row r="231" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A231" t="s">
-        <v>253</v>
+        <v>247</v>
       </c>
       <c r="B231" t="s">
-        <v>256</v>
+        <v>251</v>
       </c>
       <c r="C231">
         <v>2017</v>
       </c>
       <c r="D231" t="s">
-        <v>257</v>
+        <v>252</v>
       </c>
     </row>
     <row r="232" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A232" t="s">
-        <v>254</v>
+        <v>248</v>
       </c>
       <c r="B232" t="s">
-        <v>256</v>
+        <v>251</v>
       </c>
       <c r="C232">
         <v>2017</v>
       </c>
       <c r="D232" t="s">
-        <v>257</v>
+        <v>252</v>
       </c>
     </row>
     <row r="233" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A233" t="s">
-        <v>255</v>
+        <v>249</v>
       </c>
       <c r="B233" t="s">
-        <v>256</v>
+        <v>251</v>
       </c>
       <c r="C233">
         <v>2017</v>
       </c>
       <c r="D233" t="s">
-        <v>257</v>
+        <v>252</v>
       </c>
     </row>
     <row r="234" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A234" t="s">
-        <v>261</v>
+        <v>250</v>
       </c>
       <c r="B234" t="s">
-        <v>262</v>
+        <v>251</v>
       </c>
       <c r="C234">
-        <v>2023</v>
+        <v>2017</v>
       </c>
       <c r="D234" t="s">
-        <v>274</v>
+        <v>252</v>
       </c>
     </row>
     <row r="235" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A235" t="s">
-        <v>263</v>
+        <v>256</v>
       </c>
       <c r="B235" t="s">
-        <v>262</v>
+        <v>257</v>
       </c>
       <c r="C235">
         <v>2023</v>
       </c>
       <c r="D235" t="s">
-        <v>275</v>
+        <v>269</v>
       </c>
     </row>
     <row r="236" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A236" t="s">
-        <v>264</v>
+        <v>258</v>
       </c>
       <c r="B236" t="s">
-        <v>262</v>
+        <v>257</v>
       </c>
       <c r="C236">
         <v>2023</v>
       </c>
       <c r="D236" t="s">
-        <v>276</v>
+        <v>270</v>
       </c>
     </row>
     <row r="237" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A237" t="s">
-        <v>265</v>
+        <v>259</v>
       </c>
       <c r="B237" t="s">
-        <v>262</v>
+        <v>257</v>
       </c>
       <c r="C237">
         <v>2023</v>
       </c>
       <c r="D237" t="s">
-        <v>276</v>
+        <v>271</v>
       </c>
     </row>
     <row r="238" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A238" t="s">
-        <v>266</v>
+        <v>260</v>
       </c>
       <c r="B238" t="s">
-        <v>262</v>
+        <v>257</v>
       </c>
       <c r="C238">
         <v>2023</v>
       </c>
       <c r="D238" t="s">
-        <v>276</v>
+        <v>271</v>
       </c>
     </row>
     <row r="239" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A239" t="s">
-        <v>267</v>
+        <v>261</v>
       </c>
       <c r="B239" t="s">
-        <v>262</v>
+        <v>257</v>
       </c>
       <c r="C239">
         <v>2023</v>
       </c>
       <c r="D239" t="s">
-        <v>274</v>
+        <v>271</v>
       </c>
     </row>
     <row r="240" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A240" t="s">
-        <v>268</v>
+        <v>262</v>
       </c>
       <c r="B240" t="s">
-        <v>262</v>
+        <v>257</v>
       </c>
       <c r="C240">
         <v>2023</v>
       </c>
       <c r="D240" t="s">
-        <v>276</v>
+        <v>269</v>
       </c>
     </row>
     <row r="241" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A241" t="s">
-        <v>269</v>
+        <v>263</v>
       </c>
       <c r="B241" t="s">
-        <v>262</v>
+        <v>257</v>
       </c>
       <c r="C241">
         <v>2023</v>
       </c>
       <c r="D241" t="s">
-        <v>277</v>
+        <v>271</v>
       </c>
     </row>
     <row r="242" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A242" t="s">
-        <v>270</v>
+        <v>264</v>
       </c>
       <c r="B242" t="s">
-        <v>262</v>
+        <v>257</v>
       </c>
       <c r="C242">
         <v>2023</v>
       </c>
       <c r="D242" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
     </row>
     <row r="243" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A243" t="s">
-        <v>271</v>
+        <v>265</v>
       </c>
       <c r="B243" t="s">
-        <v>262</v>
+        <v>257</v>
       </c>
       <c r="C243">
         <v>2023</v>
       </c>
       <c r="D243" t="s">
-        <v>274</v>
+        <v>269</v>
       </c>
     </row>
     <row r="244" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A244" t="s">
-        <v>272</v>
+        <v>266</v>
       </c>
       <c r="B244" t="s">
-        <v>262</v>
+        <v>257</v>
       </c>
       <c r="C244">
         <v>2023</v>
       </c>
       <c r="D244" t="s">
-        <v>274</v>
+        <v>269</v>
       </c>
     </row>
     <row r="245" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A245" t="s">
-        <v>273</v>
+        <v>267</v>
       </c>
       <c r="B245" t="s">
-        <v>262</v>
+        <v>257</v>
       </c>
       <c r="C245">
         <v>2023</v>
       </c>
       <c r="D245" t="s">
-        <v>278</v>
+        <v>269</v>
+      </c>
+    </row>
+    <row r="246" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A246" t="s">
+        <v>268</v>
+      </c>
+      <c r="B246" t="s">
+        <v>257</v>
+      </c>
+      <c r="C246">
+        <v>2023</v>
+      </c>
+      <c r="D246" t="s">
+        <v>273</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fixed year in one of the depeche songs
</commit_message>
<xml_diff>
--- a/data/Depeche Mode Songs.xlsx
+++ b/data/Depeche Mode Songs.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lindanakasone/Documents/GitHub/sound-and-vision/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C130FD26-6901-9B41-A01B-A47793A01205}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBC5D295-6979-4D4C-A9B9-57D7C328F5D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8820" yWindow="3620" windowWidth="28040" windowHeight="22780" xr2:uid="{FE581154-A771-454D-BC0C-F4CC813A6F29}"/>
+    <workbookView xWindow="3080" yWindow="3120" windowWidth="28040" windowHeight="22780" xr2:uid="{FE581154-A771-454D-BC0C-F4CC813A6F29}"/>
   </bookViews>
   <sheets>
     <sheet name="Depeche Mode Songs" sheetId="1" r:id="rId1"/>
@@ -3287,7 +3287,7 @@
         <v>117</v>
       </c>
       <c r="C110">
-        <v>1989</v>
+        <v>1990</v>
       </c>
       <c r="D110" t="s">
         <v>118</v>

</xml_diff>